<commit_message>
Add new Excel output file COID_4981_20261021_144440.xlsx with initial data
</commit_message>
<xml_diff>
--- a/COID/Export/Production Plan_2026-10-21.xlsx
+++ b/COID/Export/Production Plan_2026-10-21.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nestle-my.sharepoint.com/personal/emmanuel_jompe_ng_nestle_com/Documents/Documents/All_Locations_for Emmanuel/COID/Export/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_D7AA1E9E0EF5F16AAB4F7373FA452B2E9310940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA783279-4CEC-4100-93A6-B6FE69E63AE9}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_D7BC66DF1F9F51E2BE13F1F4028724F09210940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5268815-ABC3-403B-AC78-FC868EAAD861}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2597" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2645" uniqueCount="221">
   <si>
     <t>PRODUCTION PLAN vs ACHIEVED (WTD) (Tons)</t>
   </si>
@@ -463,9 +463,6 @@
   </si>
   <si>
     <t>43553423</t>
-  </si>
-  <si>
-    <t>CRTD PRC  CSER BCRQ EXPL EXTS MANC SETC</t>
   </si>
   <si>
     <t>MAGGI Chicken Cube 5.5% Pre-blend NG</t>
@@ -965,7 +962,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-94BE-44FD-8C0E-33B197C59964}"/>
+              <c16:uniqueId val="{00000000-90FD-4730-937D-4E09700D981F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1009,7 +1006,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-94BE-44FD-8C0E-33B197C59964}"/>
+                <c16:uniqueId val="{00000002-90FD-4730-937D-4E09700D981F}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1027,7 +1024,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000004-94BE-44FD-8C0E-33B197C59964}"/>
+                <c16:uniqueId val="{00000004-90FD-4730-937D-4E09700D981F}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1045,7 +1042,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000006-94BE-44FD-8C0E-33B197C59964}"/>
+                <c16:uniqueId val="{00000006-90FD-4730-937D-4E09700D981F}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1063,7 +1060,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000008-94BE-44FD-8C0E-33B197C59964}"/>
+                <c16:uniqueId val="{00000008-90FD-4730-937D-4E09700D981F}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1081,7 +1078,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000A-94BE-44FD-8C0E-33B197C59964}"/>
+                <c16:uniqueId val="{0000000A-90FD-4730-937D-4E09700D981F}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1099,7 +1096,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000C-94BE-44FD-8C0E-33B197C59964}"/>
+                <c16:uniqueId val="{0000000C-90FD-4730-937D-4E09700D981F}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1117,7 +1114,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000E-94BE-44FD-8C0E-33B197C59964}"/>
+                <c16:uniqueId val="{0000000E-90FD-4730-937D-4E09700D981F}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1218,7 +1215,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000F-94BE-44FD-8C0E-33B197C59964}"/>
+              <c16:uniqueId val="{0000000F-90FD-4730-937D-4E09700D981F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1464,7 +1461,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-ECB9-48DD-8333-38DB193E1A3B}"/>
+              <c16:uniqueId val="{00000000-BBF8-4E9D-BEB1-D5D4B3F93B83}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1508,7 +1505,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-ECB9-48DD-8333-38DB193E1A3B}"/>
+                <c16:uniqueId val="{00000002-BBF8-4E9D-BEB1-D5D4B3F93B83}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1526,7 +1523,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000004-ECB9-48DD-8333-38DB193E1A3B}"/>
+                <c16:uniqueId val="{00000004-BBF8-4E9D-BEB1-D5D4B3F93B83}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1544,7 +1541,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000006-ECB9-48DD-8333-38DB193E1A3B}"/>
+                <c16:uniqueId val="{00000006-BBF8-4E9D-BEB1-D5D4B3F93B83}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1562,7 +1559,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000008-ECB9-48DD-8333-38DB193E1A3B}"/>
+                <c16:uniqueId val="{00000008-BBF8-4E9D-BEB1-D5D4B3F93B83}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1580,7 +1577,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000A-ECB9-48DD-8333-38DB193E1A3B}"/>
+                <c16:uniqueId val="{0000000A-BBF8-4E9D-BEB1-D5D4B3F93B83}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1669,7 +1666,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-ECB9-48DD-8333-38DB193E1A3B}"/>
+              <c16:uniqueId val="{0000000B-BBF8-4E9D-BEB1-D5D4B3F93B83}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1891,7 +1888,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8610-42E3-966D-C18CFD62AD2D}"/>
+              <c16:uniqueId val="{00000000-3529-4987-97A4-9EA255F87BC1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1935,7 +1932,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-8610-42E3-966D-C18CFD62AD2D}"/>
+                <c16:uniqueId val="{00000002-3529-4987-97A4-9EA255F87BC1}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -2000,7 +1997,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-8610-42E3-966D-C18CFD62AD2D}"/>
+              <c16:uniqueId val="{00000003-3529-4987-97A4-9EA255F87BC1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2222,7 +2219,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DA28-4921-9ED7-6E892414FF39}"/>
+              <c16:uniqueId val="{00000000-A14C-4CE5-BC02-8CCA72913E10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2266,7 +2263,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-DA28-4921-9ED7-6E892414FF39}"/>
+                <c16:uniqueId val="{00000002-A14C-4CE5-BC02-8CCA72913E10}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -2331,7 +2328,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-DA28-4921-9ED7-6E892414FF39}"/>
+              <c16:uniqueId val="{00000003-A14C-4CE5-BC02-8CCA72913E10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2559,7 +2556,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9CFD-4298-B4F0-F54917740619}"/>
+              <c16:uniqueId val="{00000000-33BE-47AE-A811-C89CDD3AA754}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2603,7 +2600,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-9CFD-4298-B4F0-F54917740619}"/>
+                <c16:uniqueId val="{00000002-33BE-47AE-A811-C89CDD3AA754}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -2621,7 +2618,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000004-9CFD-4298-B4F0-F54917740619}"/>
+                <c16:uniqueId val="{00000004-33BE-47AE-A811-C89CDD3AA754}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -2692,7 +2689,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-9CFD-4298-B4F0-F54917740619}"/>
+              <c16:uniqueId val="{00000005-33BE-47AE-A811-C89CDD3AA754}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2914,7 +2911,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8785-457A-B674-4897051B4F0F}"/>
+              <c16:uniqueId val="{00000000-B608-4A95-B956-73BB94AB4017}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2958,7 +2955,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-8785-457A-B674-4897051B4F0F}"/>
+                <c16:uniqueId val="{00000002-B608-4A95-B956-73BB94AB4017}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3023,7 +3020,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-8785-457A-B674-4897051B4F0F}"/>
+              <c16:uniqueId val="{00000003-B608-4A95-B956-73BB94AB4017}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3245,7 +3242,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2E33-4970-8FD7-1042F4177235}"/>
+              <c16:uniqueId val="{00000000-90FD-4A77-9F20-DEEFC3C3CDEF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3289,7 +3286,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-2E33-4970-8FD7-1042F4177235}"/>
+                <c16:uniqueId val="{00000002-90FD-4A77-9F20-DEEFC3C3CDEF}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3354,7 +3351,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-2E33-4970-8FD7-1042F4177235}"/>
+              <c16:uniqueId val="{00000003-90FD-4A77-9F20-DEEFC3C3CDEF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3680,7 +3677,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jompe,Emmanuel,NG-Sagamu, Ogun State" refreshedDate="46316.607784027779" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="84" xr:uid="{AEA8FA02-C731-4393-9D5B-9DB873CE0DBE}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jompe,Emmanuel,NG-Sagamu, Ogun State" refreshedDate="46316.629568634256" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="84" xr:uid="{9577ED40-7112-4D61-A8E5-EEB99DC5BB31}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P85" sheet="Pivot_Source"/>
   </cacheSource>
@@ -4750,7 +4747,7 @@
     <s v="KG"/>
     <x v="0"/>
     <s v="2026-10-20 00:00:00"/>
-    <s v="CRTD PRC  CSER BCRQ EXPL EXTS MANC SETC"/>
+    <s v="CRTD MSPT PRC  CSER BCRQ EXPL EXTS SETC"/>
     <x v="18"/>
     <n v="0"/>
     <s v="HALB"/>
@@ -5320,11 +5317,11 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C86D6603-11EB-4D4A-8CF8-0671BE7974FE}" name="COIDWtdPivot" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A5:C7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{27DF12EA-7E57-4CBF-B753-A346C82530D0}" name="COIDWtdPivot" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A4:D30" firstHeaderRow="1" firstDataRow="2" firstDataCol="2" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="16">
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
       <items count="25">
         <item x="0"/>
         <item x="1"/>
@@ -5373,7 +5370,7 @@
     </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
       <items count="25">
         <item x="18"/>
         <item x="13"/>
@@ -5408,8 +5405,111 @@
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
   </pivotFields>
-  <rowItems count="1">
-    <i/>
+  <rowFields count="2">
+    <field x="1"/>
+    <field x="10"/>
+  </rowFields>
+  <rowItems count="25">
+    <i>
+      <x/>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="2"/>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="3"/>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="4"/>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="5"/>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="6"/>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="7"/>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="8"/>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="10"/>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="11"/>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="12"/>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="13"/>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="14"/>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="15"/>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="16"/>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="17"/>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="18"/>
+      <x/>
+    </i>
+    <i>
+      <x v="19"/>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="20"/>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="21"/>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="22"/>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="23"/>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="24"/>
+      <x v="11"/>
+    </i>
   </rowItems>
   <colFields count="1">
     <field x="7"/>
@@ -5422,10 +5522,8 @@
       <x v="1"/>
     </i>
   </colItems>
-  <pageFields count="3">
+  <pageFields count="1">
     <pageField fld="2" hier="-1"/>
-    <pageField fld="10" hier="-1"/>
-    <pageField fld="1" hier="-1"/>
   </pageFields>
   <dataFields count="1">
     <dataField name="Sum of Delivered Quantity" fld="11" baseField="0" baseItem="0"/>
@@ -5782,61 +5880,372 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A2:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="C4" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
       <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9">
+        <v>2102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>221</v>
-      </c>
-      <c r="B7" s="9">
-        <v>698595</v>
-      </c>
-      <c r="C7" s="9">
-        <v>729665.3</v>
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9">
+        <v>9689</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="9">
+        <v>2982</v>
+      </c>
+      <c r="D10" s="9">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9">
+        <v>2082</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="9">
+        <v>0</v>
+      </c>
+      <c r="D12" s="9"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="9">
+        <v>2160</v>
+      </c>
+      <c r="D13" s="9">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="9">
+        <v>0</v>
+      </c>
+      <c r="D14" s="9"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="9">
+        <v>2340</v>
+      </c>
+      <c r="D15" s="9">
+        <v>3150</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="9">
+        <v>1764</v>
+      </c>
+      <c r="D16" s="9">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="9">
+        <v>11920</v>
+      </c>
+      <c r="D17" s="9">
+        <v>10880</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" s="9">
+        <v>1260</v>
+      </c>
+      <c r="D18" s="9">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="9">
+        <v>3180</v>
+      </c>
+      <c r="D19" s="9">
+        <v>3060</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" s="9">
+        <v>0</v>
+      </c>
+      <c r="D20" s="9">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" s="9">
+        <v>1280</v>
+      </c>
+      <c r="D21" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="9">
+        <v>16720</v>
+      </c>
+      <c r="D22" s="9">
+        <v>18160</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" t="s">
+        <v>137</v>
+      </c>
+      <c r="C23" s="9">
+        <v>0</v>
+      </c>
+      <c r="D23" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>142</v>
+      </c>
+      <c r="B24" t="s">
+        <v>143</v>
+      </c>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>145</v>
+      </c>
+      <c r="B25" t="s">
+        <v>146</v>
+      </c>
+      <c r="C25" s="9">
+        <v>3252</v>
+      </c>
+      <c r="D25" s="9"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B26" t="s">
+        <v>149</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>151</v>
+      </c>
+      <c r="B27" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" s="9">
+        <v>10854.4</v>
+      </c>
+      <c r="D27" s="9">
+        <v>10176</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>156</v>
+      </c>
+      <c r="B28" t="s">
+        <v>158</v>
+      </c>
+      <c r="C28" s="9">
+        <v>280301</v>
+      </c>
+      <c r="D28" s="9">
+        <v>366824.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B29" t="s">
+        <v>168</v>
+      </c>
+      <c r="C29" s="9">
+        <v>76300</v>
+      </c>
+      <c r="D29" s="9"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>173</v>
+      </c>
+      <c r="B30" t="s">
+        <v>174</v>
+      </c>
+      <c r="C30" s="9">
+        <v>284281.60000000003</v>
+      </c>
+      <c r="D30" s="9">
+        <v>292972.79999999999</v>
       </c>
     </row>
   </sheetData>
@@ -8354,10 +8763,10 @@
         <v>25</v>
       </c>
       <c r="J54" t="s">
+        <v>69</v>
+      </c>
+      <c r="K54" t="s">
         <v>143</v>
-      </c>
-      <c r="K54" t="s">
-        <v>144</v>
       </c>
       <c r="L54">
         <v>0</v>
@@ -8374,10 +8783,10 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>144</v>
+      </c>
+      <c r="B55" t="s">
         <v>145</v>
-      </c>
-      <c r="B55" t="s">
-        <v>146</v>
       </c>
       <c r="C55" t="s">
         <v>56</v>
@@ -8404,7 +8813,7 @@
         <v>79</v>
       </c>
       <c r="K55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L55">
         <v>3252</v>
@@ -8421,10 +8830,10 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>147</v>
+      </c>
+      <c r="B56" t="s">
         <v>148</v>
-      </c>
-      <c r="B56" t="s">
-        <v>149</v>
       </c>
       <c r="C56" t="s">
         <v>56</v>
@@ -8451,7 +8860,7 @@
         <v>64</v>
       </c>
       <c r="K56" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L56">
         <v>2100</v>
@@ -8468,10 +8877,10 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>150</v>
+      </c>
+      <c r="B57" t="s">
         <v>151</v>
-      </c>
-      <c r="B57" t="s">
-        <v>152</v>
       </c>
       <c r="C57" t="s">
         <v>56</v>
@@ -8498,7 +8907,7 @@
         <v>79</v>
       </c>
       <c r="K57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L57">
         <v>10854.4</v>
@@ -8515,10 +8924,10 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B58" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C58" t="s">
         <v>56</v>
@@ -8542,10 +8951,10 @@
         <v>25</v>
       </c>
       <c r="J58" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K58" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L58">
         <v>10176</v>
@@ -8562,10 +8971,10 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>155</v>
+      </c>
+      <c r="B59" t="s">
         <v>156</v>
-      </c>
-      <c r="B59" t="s">
-        <v>157</v>
       </c>
       <c r="C59" t="s">
         <v>56</v>
@@ -8589,10 +8998,10 @@
         <v>58</v>
       </c>
       <c r="J59" t="s">
+        <v>157</v>
+      </c>
+      <c r="K59" t="s">
         <v>158</v>
-      </c>
-      <c r="K59" t="s">
-        <v>159</v>
       </c>
       <c r="L59">
         <v>0</v>
@@ -8609,10 +9018,10 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B60" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C60" t="s">
         <v>56</v>
@@ -8639,7 +9048,7 @@
         <v>64</v>
       </c>
       <c r="K60" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L60">
         <v>280301</v>
@@ -8656,10 +9065,10 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B61" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C61" t="s">
         <v>95</v>
@@ -8680,10 +9089,10 @@
         <v>48</v>
       </c>
       <c r="I61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K61" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L61">
         <v>0</v>
@@ -8700,10 +9109,10 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B62" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C62" t="s">
         <v>56</v>
@@ -8730,7 +9139,7 @@
         <v>64</v>
       </c>
       <c r="K62" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L62">
         <v>256346</v>
@@ -8747,10 +9156,10 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B63" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C63" t="s">
         <v>56</v>
@@ -8777,7 +9186,7 @@
         <v>64</v>
       </c>
       <c r="K63" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L63">
         <v>87943</v>
@@ -8794,10 +9203,10 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B64" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C64" t="s">
         <v>56</v>
@@ -8824,7 +9233,7 @@
         <v>64</v>
       </c>
       <c r="K64" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L64">
         <v>22535.5</v>
@@ -8841,10 +9250,10 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>165</v>
+      </c>
+      <c r="B65" t="s">
         <v>166</v>
-      </c>
-      <c r="B65" t="s">
-        <v>167</v>
       </c>
       <c r="C65" t="s">
         <v>56</v>
@@ -8868,10 +9277,10 @@
         <v>58</v>
       </c>
       <c r="J65" t="s">
+        <v>167</v>
+      </c>
+      <c r="K65" t="s">
         <v>168</v>
-      </c>
-      <c r="K65" t="s">
-        <v>169</v>
       </c>
       <c r="L65">
         <v>0</v>
@@ -8888,10 +9297,10 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B66" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C66" t="s">
         <v>56</v>
@@ -8918,7 +9327,7 @@
         <v>64</v>
       </c>
       <c r="K66" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L66">
         <v>76300</v>
@@ -8935,10 +9344,10 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B67" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C67" t="s">
         <v>95</v>
@@ -8959,10 +9368,10 @@
         <v>48</v>
       </c>
       <c r="I67" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K67" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L67">
         <v>0</v>
@@ -8979,10 +9388,10 @@
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>172</v>
+      </c>
+      <c r="B68" t="s">
         <v>173</v>
-      </c>
-      <c r="B68" t="s">
-        <v>174</v>
       </c>
       <c r="C68" t="s">
         <v>56</v>
@@ -9009,7 +9418,7 @@
         <v>64</v>
       </c>
       <c r="K68" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L68">
         <v>16960</v>
@@ -9026,10 +9435,10 @@
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B69" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C69" t="s">
         <v>56</v>
@@ -9056,7 +9465,7 @@
         <v>64</v>
       </c>
       <c r="K69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L69">
         <v>77536</v>
@@ -9073,10 +9482,10 @@
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B70" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C70" t="s">
         <v>56</v>
@@ -9103,7 +9512,7 @@
         <v>64</v>
       </c>
       <c r="K70" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L70">
         <v>70537.600000000006</v>
@@ -9120,10 +9529,10 @@
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B71" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C71" t="s">
         <v>56</v>
@@ -9150,7 +9559,7 @@
         <v>64</v>
       </c>
       <c r="K71" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L71">
         <v>13267.2</v>
@@ -9167,10 +9576,10 @@
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B72" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C72" t="s">
         <v>56</v>
@@ -9197,7 +9606,7 @@
         <v>64</v>
       </c>
       <c r="K72" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L72">
         <v>75792</v>
@@ -9214,10 +9623,10 @@
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B73" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C73" t="s">
         <v>56</v>
@@ -9244,7 +9653,7 @@
         <v>64</v>
       </c>
       <c r="K73" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L73">
         <v>30188.799999999999</v>
@@ -9261,10 +9670,10 @@
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B74" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C74" t="s">
         <v>56</v>
@@ -9291,7 +9700,7 @@
         <v>69</v>
       </c>
       <c r="K74" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L74">
         <v>0</v>
@@ -9308,10 +9717,10 @@
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B75" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C75" t="s">
         <v>95</v>
@@ -9335,7 +9744,7 @@
         <v>58</v>
       </c>
       <c r="K75" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L75">
         <v>0</v>
@@ -9352,10 +9761,10 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B76" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C76" t="s">
         <v>56</v>
@@ -9379,10 +9788,10 @@
         <v>39</v>
       </c>
       <c r="J76" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K76" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L76">
         <v>79696</v>
@@ -9399,10 +9808,10 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B77" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C77" t="s">
         <v>56</v>
@@ -9426,10 +9835,10 @@
         <v>39</v>
       </c>
       <c r="J77" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K77" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L77">
         <v>80806.399999999994</v>
@@ -9446,10 +9855,10 @@
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B78" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C78" t="s">
         <v>56</v>
@@ -9473,10 +9882,10 @@
         <v>39</v>
       </c>
       <c r="J78" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K78" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L78">
         <v>15798.4</v>
@@ -9493,10 +9902,10 @@
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B79" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C79" t="s">
         <v>56</v>
@@ -9520,10 +9929,10 @@
         <v>25</v>
       </c>
       <c r="J79" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K79" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L79">
         <v>31206.400000000001</v>
@@ -9540,10 +9949,10 @@
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B80" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C80" t="s">
         <v>56</v>
@@ -9567,10 +9976,10 @@
         <v>25</v>
       </c>
       <c r="J80" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K80" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L80">
         <v>68166.399999999994</v>
@@ -9587,10 +9996,10 @@
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B81" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C81" t="s">
         <v>56</v>
@@ -9617,7 +10026,7 @@
         <v>69</v>
       </c>
       <c r="K81" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L81">
         <v>0</v>
@@ -9634,10 +10043,10 @@
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B82" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C82" t="s">
         <v>56</v>
@@ -9664,7 +10073,7 @@
         <v>69</v>
       </c>
       <c r="K82" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L82">
         <v>0</v>
@@ -9681,10 +10090,10 @@
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B83" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C83" t="s">
         <v>56</v>
@@ -9711,7 +10120,7 @@
         <v>69</v>
       </c>
       <c r="K83" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L83">
         <v>0</v>
@@ -9728,10 +10137,10 @@
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B84" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C84" t="s">
         <v>56</v>
@@ -9758,7 +10167,7 @@
         <v>69</v>
       </c>
       <c r="K84" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L84">
         <v>0</v>
@@ -9775,10 +10184,10 @@
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B85" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C85" t="s">
         <v>56</v>
@@ -9802,10 +10211,10 @@
         <v>39</v>
       </c>
       <c r="J85" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K85" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L85">
         <v>17299.2</v>
@@ -12336,10 +12745,10 @@
         <v>25</v>
       </c>
       <c r="J54" t="s">
+        <v>69</v>
+      </c>
+      <c r="K54" t="s">
         <v>143</v>
-      </c>
-      <c r="K54" t="s">
-        <v>144</v>
       </c>
       <c r="L54">
         <v>0</v>
@@ -12356,10 +12765,10 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>144</v>
+      </c>
+      <c r="B55" t="s">
         <v>145</v>
-      </c>
-      <c r="B55" t="s">
-        <v>146</v>
       </c>
       <c r="C55" t="s">
         <v>56</v>
@@ -12386,7 +12795,7 @@
         <v>79</v>
       </c>
       <c r="K55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L55">
         <v>3252</v>
@@ -12403,10 +12812,10 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>147</v>
+      </c>
+      <c r="B56" t="s">
         <v>148</v>
-      </c>
-      <c r="B56" t="s">
-        <v>149</v>
       </c>
       <c r="C56" t="s">
         <v>56</v>
@@ -12433,7 +12842,7 @@
         <v>64</v>
       </c>
       <c r="K56" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L56">
         <v>2100</v>
@@ -12450,10 +12859,10 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>150</v>
+      </c>
+      <c r="B57" t="s">
         <v>151</v>
-      </c>
-      <c r="B57" t="s">
-        <v>152</v>
       </c>
       <c r="C57" t="s">
         <v>56</v>
@@ -12480,7 +12889,7 @@
         <v>79</v>
       </c>
       <c r="K57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L57">
         <v>10854.4</v>
@@ -12497,10 +12906,10 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B58" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C58" t="s">
         <v>56</v>
@@ -12524,10 +12933,10 @@
         <v>25</v>
       </c>
       <c r="J58" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K58" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L58">
         <v>10176</v>
@@ -12544,10 +12953,10 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>155</v>
+      </c>
+      <c r="B59" t="s">
         <v>156</v>
-      </c>
-      <c r="B59" t="s">
-        <v>157</v>
       </c>
       <c r="C59" t="s">
         <v>56</v>
@@ -12571,10 +12980,10 @@
         <v>58</v>
       </c>
       <c r="J59" t="s">
+        <v>157</v>
+      </c>
+      <c r="K59" t="s">
         <v>158</v>
-      </c>
-      <c r="K59" t="s">
-        <v>159</v>
       </c>
       <c r="L59">
         <v>0</v>
@@ -12591,10 +13000,10 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B60" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C60" t="s">
         <v>56</v>
@@ -12621,7 +13030,7 @@
         <v>64</v>
       </c>
       <c r="K60" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L60">
         <v>280301</v>
@@ -12638,10 +13047,10 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B61" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C61" t="s">
         <v>95</v>
@@ -12662,10 +13071,10 @@
         <v>48</v>
       </c>
       <c r="I61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K61" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L61">
         <v>0</v>
@@ -12682,10 +13091,10 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B62" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C62" t="s">
         <v>56</v>
@@ -12712,7 +13121,7 @@
         <v>64</v>
       </c>
       <c r="K62" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L62">
         <v>256346</v>
@@ -12729,10 +13138,10 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B63" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C63" t="s">
         <v>56</v>
@@ -12759,7 +13168,7 @@
         <v>64</v>
       </c>
       <c r="K63" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L63">
         <v>87943</v>
@@ -12776,10 +13185,10 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B64" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C64" t="s">
         <v>56</v>
@@ -12806,7 +13215,7 @@
         <v>64</v>
       </c>
       <c r="K64" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L64">
         <v>22535.5</v>
@@ -12823,10 +13232,10 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>165</v>
+      </c>
+      <c r="B65" t="s">
         <v>166</v>
-      </c>
-      <c r="B65" t="s">
-        <v>167</v>
       </c>
       <c r="C65" t="s">
         <v>56</v>
@@ -12850,10 +13259,10 @@
         <v>58</v>
       </c>
       <c r="J65" t="s">
+        <v>167</v>
+      </c>
+      <c r="K65" t="s">
         <v>168</v>
-      </c>
-      <c r="K65" t="s">
-        <v>169</v>
       </c>
       <c r="L65">
         <v>0</v>
@@ -12870,10 +13279,10 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B66" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C66" t="s">
         <v>56</v>
@@ -12900,7 +13309,7 @@
         <v>64</v>
       </c>
       <c r="K66" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L66">
         <v>76300</v>
@@ -12917,10 +13326,10 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B67" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C67" t="s">
         <v>95</v>
@@ -12941,10 +13350,10 @@
         <v>48</v>
       </c>
       <c r="I67" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K67" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L67">
         <v>0</v>
@@ -12961,10 +13370,10 @@
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>172</v>
+      </c>
+      <c r="B68" t="s">
         <v>173</v>
-      </c>
-      <c r="B68" t="s">
-        <v>174</v>
       </c>
       <c r="C68" t="s">
         <v>56</v>
@@ -12991,7 +13400,7 @@
         <v>64</v>
       </c>
       <c r="K68" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L68">
         <v>16960</v>
@@ -13008,10 +13417,10 @@
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B69" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C69" t="s">
         <v>56</v>
@@ -13038,7 +13447,7 @@
         <v>64</v>
       </c>
       <c r="K69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L69">
         <v>77536</v>
@@ -13055,10 +13464,10 @@
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B70" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C70" t="s">
         <v>56</v>
@@ -13085,7 +13494,7 @@
         <v>64</v>
       </c>
       <c r="K70" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L70">
         <v>70537.600000000006</v>
@@ -13102,10 +13511,10 @@
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B71" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C71" t="s">
         <v>56</v>
@@ -13132,7 +13541,7 @@
         <v>64</v>
       </c>
       <c r="K71" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L71">
         <v>13267.2</v>
@@ -13149,10 +13558,10 @@
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B72" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C72" t="s">
         <v>56</v>
@@ -13179,7 +13588,7 @@
         <v>64</v>
       </c>
       <c r="K72" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L72">
         <v>75792</v>
@@ -13196,10 +13605,10 @@
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B73" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C73" t="s">
         <v>56</v>
@@ -13226,7 +13635,7 @@
         <v>64</v>
       </c>
       <c r="K73" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L73">
         <v>30188.799999999999</v>
@@ -13243,10 +13652,10 @@
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B74" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C74" t="s">
         <v>56</v>
@@ -13273,7 +13682,7 @@
         <v>69</v>
       </c>
       <c r="K74" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L74">
         <v>0</v>
@@ -13290,10 +13699,10 @@
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B75" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C75" t="s">
         <v>95</v>
@@ -13317,7 +13726,7 @@
         <v>58</v>
       </c>
       <c r="K75" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L75">
         <v>0</v>
@@ -13334,10 +13743,10 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B76" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C76" t="s">
         <v>56</v>
@@ -13361,10 +13770,10 @@
         <v>39</v>
       </c>
       <c r="J76" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K76" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L76">
         <v>79696</v>
@@ -13381,10 +13790,10 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B77" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C77" t="s">
         <v>56</v>
@@ -13408,10 +13817,10 @@
         <v>39</v>
       </c>
       <c r="J77" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K77" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L77">
         <v>80806.399999999994</v>
@@ -13428,10 +13837,10 @@
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B78" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C78" t="s">
         <v>56</v>
@@ -13455,10 +13864,10 @@
         <v>39</v>
       </c>
       <c r="J78" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K78" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L78">
         <v>15798.4</v>
@@ -13475,10 +13884,10 @@
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B79" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C79" t="s">
         <v>56</v>
@@ -13502,10 +13911,10 @@
         <v>25</v>
       </c>
       <c r="J79" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K79" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L79">
         <v>31206.400000000001</v>
@@ -13522,10 +13931,10 @@
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B80" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C80" t="s">
         <v>56</v>
@@ -13549,10 +13958,10 @@
         <v>25</v>
       </c>
       <c r="J80" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K80" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L80">
         <v>68166.399999999994</v>
@@ -13569,10 +13978,10 @@
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B81" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C81" t="s">
         <v>56</v>
@@ -13599,7 +14008,7 @@
         <v>69</v>
       </c>
       <c r="K81" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L81">
         <v>0</v>
@@ -13616,10 +14025,10 @@
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B82" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C82" t="s">
         <v>56</v>
@@ -13646,7 +14055,7 @@
         <v>69</v>
       </c>
       <c r="K82" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L82">
         <v>0</v>
@@ -13663,10 +14072,10 @@
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B83" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C83" t="s">
         <v>56</v>
@@ -13693,7 +14102,7 @@
         <v>69</v>
       </c>
       <c r="K83" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L83">
         <v>0</v>
@@ -13710,10 +14119,10 @@
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B84" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C84" t="s">
         <v>56</v>
@@ -13740,7 +14149,7 @@
         <v>69</v>
       </c>
       <c r="K84" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L84">
         <v>0</v>
@@ -13757,10 +14166,10 @@
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B85" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C85" t="s">
         <v>56</v>
@@ -13784,10 +14193,10 @@
         <v>39</v>
       </c>
       <c r="J85" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K85" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L85">
         <v>17299.2</v>
@@ -13814,72 +14223,72 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B1" t="s">
         <v>193</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>194</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>195</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>196</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>197</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>198</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>199</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>200</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>201</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>202</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>203</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>204</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>205</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>206</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>207</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>208</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>209</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>210</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>211</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>212</v>
-      </c>
-      <c r="U1" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B2">
         <v>632.63900000000001</v>
@@ -13944,7 +14353,7 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B3">
         <v>1.98</v>
@@ -13973,7 +14382,7 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B4">
         <v>50</v>
@@ -13993,7 +14402,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B5">
         <v>16.32</v>
@@ -14013,7 +14422,7 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B6">
         <v>788.39800000000002</v>
@@ -14033,7 +14442,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B7">
         <v>119.85599999999999</v>
@@ -14044,7 +14453,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B8">
         <v>3</v>
@@ -14075,7 +14484,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -14090,13 +14499,13 @@
         <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -14104,10 +14513,10 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D2" t="s">
         <v>138</v>
@@ -14122,7 +14531,7 @@
         <v>280.30099999999999</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -14133,7 +14542,7 @@
         <v>142</v>
       </c>
       <c r="C3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D3" t="s">
         <v>138</v>
@@ -14148,7 +14557,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -14156,10 +14565,10 @@
         <v>48</v>
       </c>
       <c r="B4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" t="s">
         <v>149</v>
-      </c>
-      <c r="C4" t="s">
-        <v>150</v>
       </c>
       <c r="D4" t="s">
         <v>138</v>
@@ -14174,7 +14583,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -14182,10 +14591,10 @@
         <v>48</v>
       </c>
       <c r="B5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C5" t="s">
         <v>152</v>
-      </c>
-      <c r="C5" t="s">
-        <v>153</v>
       </c>
       <c r="D5" t="s">
         <v>138</v>
@@ -14200,7 +14609,7 @@
         <v>10.8544</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -14208,10 +14617,10 @@
         <v>48</v>
       </c>
       <c r="B6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C6" t="s">
         <v>174</v>
-      </c>
-      <c r="C6" t="s">
-        <v>175</v>
       </c>
       <c r="D6" t="s">
         <v>138</v>
@@ -14226,7 +14635,7 @@
         <v>284.28160000000003</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -14234,10 +14643,10 @@
         <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D7" t="s">
         <v>138</v>
@@ -14252,7 +14661,7 @@
         <v>76.3</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -14260,10 +14669,10 @@
         <v>48</v>
       </c>
       <c r="B8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C8" t="s">
         <v>146</v>
-      </c>
-      <c r="C8" t="s">
-        <v>147</v>
       </c>
       <c r="D8" t="s">
         <v>138</v>
@@ -14278,7 +14687,7 @@
         <v>3.2519999999999998</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -14304,7 +14713,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -14330,7 +14739,7 @@
         <v>141.78559999999999</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -14356,7 +14765,7 @@
         <v>109.664</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -14382,7 +14791,7 @@
         <v>21.6</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -14408,7 +14817,7 @@
         <v>11.231999999999999</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -14434,7 +14843,7 @@
         <v>10.8544</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -14460,7 +14869,7 @@
         <v>4.2336</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -14486,7 +14895,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -14512,7 +14921,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -14538,7 +14947,7 @@
         <v>18.143999999999998</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -14564,7 +14973,7 @@
         <v>22.896000000000001</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -14572,10 +14981,10 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D20" t="s">
         <v>138</v>
@@ -14590,7 +14999,7 @@
         <v>366.8245</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -14601,7 +15010,7 @@
         <v>142</v>
       </c>
       <c r="C21" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D21" t="s">
         <v>138</v>
@@ -14616,7 +15025,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -14624,10 +15033,10 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C22" t="s">
         <v>149</v>
-      </c>
-      <c r="C22" t="s">
-        <v>150</v>
       </c>
       <c r="D22" t="s">
         <v>138</v>
@@ -14642,7 +15051,7 @@
         <v>2.1</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -14650,10 +15059,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" t="s">
         <v>152</v>
-      </c>
-      <c r="C23" t="s">
-        <v>153</v>
       </c>
       <c r="D23" t="s">
         <v>138</v>
@@ -14668,7 +15077,7 @@
         <v>10.176</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -14676,10 +15085,10 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
+        <v>173</v>
+      </c>
+      <c r="C24" t="s">
         <v>174</v>
-      </c>
-      <c r="C24" t="s">
-        <v>175</v>
       </c>
       <c r="D24" t="s">
         <v>138</v>
@@ -14694,7 +15103,7 @@
         <v>292.97280000000001</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -14702,10 +15111,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D25" t="s">
         <v>138</v>
@@ -14720,7 +15129,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -14728,10 +15137,10 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
+        <v>145</v>
+      </c>
+      <c r="C26" t="s">
         <v>146</v>
-      </c>
-      <c r="C26" t="s">
-        <v>147</v>
       </c>
       <c r="D26" t="s">
         <v>138</v>
@@ -14746,7 +15155,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -14772,7 +15181,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -14798,7 +15207,7 @@
         <v>153.99680000000001</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -14824,7 +15233,7 @@
         <v>100.096</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -14850,7 +15259,7 @@
         <v>23.76</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -14876,7 +15285,7 @@
         <v>15.12</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -14902,7 +15311,7 @@
         <v>10.176</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -14928,7 +15337,7 @@
         <v>2.1168</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -14954,7 +15363,7 @@
         <v>1.8</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -14980,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -15006,7 +15415,7 @@
         <v>12.096</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -15032,7 +15441,7 @@
         <v>22.032</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -15832,10 +16241,10 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C18" t="s">
         <v>95</v>
@@ -15856,10 +16265,10 @@
         <v>48</v>
       </c>
       <c r="I18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L18">
         <v>0</v>
@@ -15876,10 +16285,10 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C19" t="s">
         <v>95</v>
@@ -15900,10 +16309,10 @@
         <v>48</v>
       </c>
       <c r="I19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L19">
         <v>0</v>
@@ -15920,10 +16329,10 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C20" t="s">
         <v>95</v>
@@ -15947,7 +16356,7 @@
         <v>58</v>
       </c>
       <c r="K20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L20">
         <v>0</v>

</xml_diff>